<commit_message>
rec pbi uta 21 jul
</commit_message>
<xml_diff>
--- a/Power BI/1. Get Data - Importar Datos/Excel/Carpeta con varios archivos de Excel (Tickets)/2023.xlsx
+++ b/Power BI/1. Get Data - Importar Datos/Excel/Carpeta con varios archivos de Excel (Tickets)/2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Empresa\Programas\Diplomados\POWER BI\Power BI - Global (Para todos los programas)\1. Get Data - Importar Datos\Excel\Carpeta con varios archivos de Excel (Tickets)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7922b0b09328d329/Data World/Programas/Data Analyst Carreer/Data Academy - Repository/Power BI/1. Get Data - Importar Datos/Excel/Carpeta con varios archivos de Excel (Tickets)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0BE28C-B0BB-47BD-89C6-70FFDD9AB3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{0C0BE28C-B0BB-47BD-89C6-70FFDD9AB3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86217EC8-061B-4BD7-86CD-CFAE81A08D21}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TicketsTI" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="26">
   <si>
     <t>Hardware</t>
   </si>
@@ -127,8 +127,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -645,7 +645,7 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -658,7 +658,7 @@
     <xf numFmtId="1" fontId="13" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -981,24 +981,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
@@ -1031,13 +1031,13 @@
       </c>
       <c r="L1"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="7">
         <f ca="1">+TODAY()</f>
-        <v>45258</v>
+        <v>45842</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>5</v>
@@ -1065,13 +1065,13 @@
       </c>
       <c r="L2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="7">
         <f ca="1">+B2+1</f>
-        <v>45259</v>
+        <v>45843</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>5</v>
@@ -1099,13 +1099,13 @@
       </c>
       <c r="L3"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="7">
-        <f t="shared" ref="B4:B10" ca="1" si="0">+B3+1</f>
-        <v>45260</v>
+        <f t="shared" ref="B4:B12" ca="1" si="0">+B3+1</f>
+        <v>45844</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>5</v>
@@ -1133,13 +1133,13 @@
       </c>
       <c r="L4"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45261</v>
+        <v>45845</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>5</v>
@@ -1167,13 +1167,13 @@
       </c>
       <c r="L5"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45262</v>
+        <v>45846</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>5</v>
@@ -1201,13 +1201,13 @@
       </c>
       <c r="L6"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45263</v>
+        <v>45847</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>5</v>
@@ -1235,13 +1235,13 @@
       </c>
       <c r="L7"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45264</v>
+        <v>45848</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>4</v>
@@ -1269,13 +1269,13 @@
       </c>
       <c r="L8"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45265</v>
+        <v>45849</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>4</v>
@@ -1303,13 +1303,13 @@
       </c>
       <c r="L9"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45266</v>
+        <v>45850</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>4</v>
@@ -1336,6 +1336,72 @@
         <v>5</v>
       </c>
       <c r="L10"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="7">
+        <f t="shared" ca="1" si="0"/>
+        <v>45851</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="6">
+        <v>1609</v>
+      </c>
+      <c r="F11" s="6">
+        <v>7</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I11" s="8">
+        <v>13</v>
+      </c>
+      <c r="J11" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="7">
+        <f t="shared" ca="1" si="0"/>
+        <v>45852</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="6">
+        <v>1609</v>
+      </c>
+      <c r="F12" s="6">
+        <v>7</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I12" s="8">
+        <v>13</v>
+      </c>
+      <c r="J12" s="8">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J10" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>